<commit_message>
feat(training): adicionar agenda semanal explicita
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/daygym-modelo-oficial-treino.xlsx
+++ b/apps/web/public/templates/daygym-modelo-oficial-treino.xlsx
@@ -28,40 +28,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tipos aceitos: força, tempo, distância, cardio e circuito.</t>
+          <t>Na coluna Dia: 1 é segunda, 2 terça, 3 quarta e assim até 7 domingo.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Força exige Reps mín e Reps máx. Tempo exige Duração (s).</t>
+          <t>Tipos aceitos: força, tempo, distância, cardio e circuito.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Distância e cardio exigem Duração (s) ou Distância (m).</t>
+          <t>Força exige Reps mín e Reps máx. Tempo exige Duração (s).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Circuito exige um nome na coluna Circuito.</t>
+          <t>Distância e cardio exigem Duração (s) ou Distância (m).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>O arquivo deve permanecer .xlsx e ter no máximo 2 MB.</t>
+          <t>Circuito exige um nome na coluna Circuito.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>O arquivo deve permanecer .xlsx e ter no máximo 2 MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Macros, fórmulas, links, proteção e objetos incorporados bloqueiam a importação.</t>
         </is>

</xml_diff>

<commit_message>
feat(training): persist workout execution by set
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/daygym-modelo-oficial-treino.xlsx
+++ b/apps/web/public/templates/daygym-modelo-oficial-treino.xlsx
@@ -63,12 +63,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>O arquivo deve permanecer .xlsx e ter no máximo 2 MB.</t>
+          <t>Carga (kg) é opcional e aceita até duas casas decimais.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>O arquivo deve permanecer .xlsx e ter no máximo 2 MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Macros, fórmulas, links, proteção e objetos incorporados bloqueiam a importação.</t>
         </is>
@@ -147,6 +154,11 @@
           <t>Observações</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Carga (kg)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -181,6 +193,9 @@
       </c>
       <c r="K2">
         <v>90</v>
+      </c>
+      <c r="N2">
+        <v>40</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
feat(web): simplify training plan experience
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/daygym-modelo-oficial-treino.xlsx
+++ b/apps/web/public/templates/daygym-modelo-oficial-treino.xlsx
@@ -42,40 +42,47 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Força exige Reps mín e Reps máx. Tempo exige Duração (s).</t>
+          <t>Força exige Reps mín e Reps máx. Tempo exige Duração (HH:MM:SS).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Distância e cardio exigem Duração (s) ou Distância (m).</t>
+          <t>Distância e cardio exigem Duração (HH:MM:SS) ou Distância (m).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Circuito exige um nome na coluna Circuito.</t>
+          <t>Exemplo de tempo: 00:30:00 representa 30 minutos.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Carga (kg) é opcional e aceita até duas casas decimais.</t>
+          <t>Circuito exige um nome na coluna Circuito.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>O arquivo deve permanecer .xlsx e ter no máximo 2 MB.</t>
+          <t>Carga (kg) é opcional e aceita até duas casas decimais.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>O arquivo deve permanecer .xlsx e ter no máximo 2 MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Macros, fórmulas, links, proteção e objetos incorporados bloqueiam a importação.</t>
         </is>
@@ -131,7 +138,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Duração (s)</t>
+          <t>Duração (HH:MM:SS)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -141,7 +148,7 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Descanso (s)</t>
+          <t>Descanso (HH:MM:SS)</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -191,8 +198,10 @@
       <c r="H2">
         <v>12</v>
       </c>
-      <c r="K2">
-        <v>90</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>00:01:30</t>
+        </is>
       </c>
       <c r="N2">
         <v>40</v>
@@ -223,11 +232,15 @@
       <c r="F3">
         <v>3</v>
       </c>
-      <c r="I3">
-        <v>30</v>
-      </c>
-      <c r="K3">
-        <v>45</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>00:00:30</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>00:00:45</t>
+        </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -260,11 +273,15 @@
       <c r="F4">
         <v>1</v>
       </c>
-      <c r="I4">
-        <v>1200</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>00:20:00</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>